<commit_message>
Diff depo, diff sett. -_-
</commit_message>
<xml_diff>
--- a/Contoh Data/Avg_temp.xlsx
+++ b/Contoh Data/Avg_temp.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\ADM IRC AND ZN\Automasi-AR-Orderan-main\Dapur\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\ADM IRC AND ZN\Automasi-AR-Orderan-IHFANDI BRANCH\Dapur\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{998E7EF6-BD8C-4E66-BDB5-6B4B370CA316}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3D79448-9BC7-48B9-A197-F060050C6CD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>AVG</t>
   </si>
@@ -63,6 +63,9 @@
   </si>
   <si>
     <t>AVG HISTORY BAYAR (HARI)</t>
+  </si>
+  <si>
+    <t>TIERING</t>
   </si>
 </sst>
 </file>
@@ -328,20 +331,19 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="27.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.5703125" customWidth="1"/>
+    <col min="2" max="2" width="43.7109375" customWidth="1"/>
+    <col min="3" max="3" width="17.5703125" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="5" max="5" width="15" customWidth="1"/>
+    <col min="7" max="7" width="18.140625" customWidth="1"/>
+    <col min="8" max="8" width="23.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -349,7 +351,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
@@ -373,6 +375,9 @@
       </c>
       <c r="H2" s="2" t="s">
         <v>9</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>